<commit_message>
Update WP8 site codes refs #1382
</commit_message>
<xml_diff>
--- a/R-dataprocessor/dataprocessor/inst/extdata/Standortkuerzel.xlsx
+++ b/R-dataprocessor/dataprocessor/inst/extdata/Standortkuerzel.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t xml:space="preserve">SITE_CODE</t>
   </si>
@@ -70,7 +70,7 @@
     <t xml:space="preserve">Universitätsklinikum Gießen</t>
   </si>
   <si>
-    <t xml:space="preserve">UKHB</t>
+    <t xml:space="preserve">UKHD</t>
   </si>
   <si>
     <t xml:space="preserve">Universitätsklinikum Heidelberg</t>
@@ -94,7 +94,7 @@
     <t xml:space="preserve">Universitätsklinikum Leipzig</t>
   </si>
   <si>
-    <t xml:space="preserve">UKM</t>
+    <t xml:space="preserve">UKMZ</t>
   </si>
   <si>
     <t xml:space="preserve">Universitätsklinikum Mainz</t>
@@ -104,6 +104,12 @@
   </si>
   <si>
     <t xml:space="preserve">Universitätsklinikum München</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UKH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Universitätsklinikum Halle (Saale)</t>
   </si>
 </sst>
 </file>
@@ -113,7 +119,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -135,6 +141,12 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -179,8 +191,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -204,34 +224,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -376,122 +396,130 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
-  <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B15"/>
+  <sheetFormatPr defaultColWidth="10.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="35.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35.19"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>